<commit_message>
Update output files: replace MailboxesWithTargetPolicy.xlsx and remove temporary migration result files
</commit_message>
<xml_diff>
--- a/Input Data/Aerotek FTE.xlsx
+++ b/Input Data/Aerotek FTE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DakotaRuhl\Documents\PS-DR\Input Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC9A4FFB-959F-495D-BB6E-0164E4CB0252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAEC695E-4B1C-4E47-85CF-0BD3D438BCB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Results" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Results!$A$1:$H$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Results!$A$1:$I$27</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -164,9 +164,6 @@
     <t>Alex Arroyo</t>
   </si>
   <si>
-    <t>aarroyo@erock.com</t>
-  </si>
-  <si>
     <t>Skipped</t>
   </si>
   <si>
@@ -365,9 +362,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Converted License from E5</t>
-  </si>
-  <si>
     <t>Complete</t>
   </si>
   <si>
@@ -381,6 +375,12 @@
   </si>
   <si>
     <t>Microsoft 365 Business Premium, Defender Suite for Business Premium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onboarding Tasks </t>
+  </si>
+  <si>
+    <t>alex.arroyo@erock.com</t>
   </si>
 </sst>
 </file>
@@ -431,7 +431,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -441,6 +441,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -459,7 +465,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -482,13 +488,22 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{09AA59FC-02FA-41E6-93ED-BE6673DCF9B5}"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="11">
     <dxf>
       <fill>
         <patternFill>
@@ -593,6 +608,24 @@
       </font>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -626,16 +659,34 @@
 </styleSheet>
 </file>
 
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{28ADF923-25A8-490F-94BB-FAF1391DF5BD}" name="Table1" displayName="Table1" ref="A1:O27" totalsRowShown="0" headerRowDxfId="9">
-  <autoFilter ref="A1:O27" xr:uid="{28ADF923-25A8-490F-94BB-FAF1391DF5BD}"/>
-  <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{E2B6BD7E-FB7C-445D-B459-13FBE42FD0A3}" name="Complete" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{28ADF923-25A8-490F-94BB-FAF1391DF5BD}" name="Table1" displayName="Table1" ref="A1:P27" totalsRowShown="0" headerRowDxfId="10">
+  <autoFilter ref="A1:P27" xr:uid="{28ADF923-25A8-490F-94BB-FAF1391DF5BD}"/>
+  <tableColumns count="16">
+    <tableColumn id="1" xr3:uid="{E2B6BD7E-FB7C-445D-B459-13FBE42FD0A3}" name="Complete" dataDxfId="9">
       <calculatedColumnFormula>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{EB9EEA4D-4A68-426F-9FA9-D933293BDCFB}" name="DisplayName"/>
     <tableColumn id="4" xr3:uid="{88E43C09-B05E-4B93-8497-F8A04D92B388}" name="UPN"/>
-    <tableColumn id="3" xr3:uid="{29720B93-12D6-445C-A769-5C8D578F4783}" name="Offboard -SC account" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{29720B93-12D6-445C-A769-5C8D578F4783}" name="Offboard -SC account" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{BA89BF43-B152-4141-8046-124F786C71A0}" name="Onboarding Tasks " dataDxfId="7"/>
     <tableColumn id="6" xr3:uid="{CBF3F29A-9850-46A1-8DB8-EB90CD7F1ED5}" name="Action"/>
     <tableColumn id="7" xr3:uid="{775C3CE4-DBB4-4963-8991-7AFD8348F168}" name="Status"/>
     <tableColumn id="8" xr3:uid="{3DE09A5F-5298-46F7-A397-80F1ACC8BA8C}" name="UserId"/>
@@ -969,27 +1020,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O27"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="3" width="23.5703125" customWidth="1"/>
     <col min="4" max="4" width="28.7109375" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" customWidth="1"/>
-    <col min="7" max="7" width="7.42578125" customWidth="1"/>
-    <col min="8" max="8" width="11" customWidth="1"/>
-    <col min="9" max="9" width="40.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" customWidth="1"/>
+    <col min="8" max="8" width="7.42578125" customWidth="1"/>
+    <col min="9" max="9" width="11" customWidth="1"/>
+    <col min="10" max="10" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="34.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -998,43 +1050,46 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="5" t="s">
-        <v>110</v>
-      </c>
       <c r="M1" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="N1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="5" t="s">
-        <v>111</v>
-      </c>
       <c r="O1" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>106</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
@@ -1046,40 +1101,43 @@
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
-      </c>
-      <c r="E2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J2" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L2" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N2" s="4" t="b">
+      <c r="K2" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O2" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
@@ -1091,40 +1149,43 @@
         <v>18</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E3" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
         <v>11</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>12</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>19</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J3" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L3" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N3" s="4" t="b">
+      <c r="K3" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M3" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
@@ -1135,41 +1196,44 @@
       <c r="C4" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="E4" s="8" t="s">
+      <c r="D4" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="E4" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="G4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="H4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="I4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="J4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="K4" s="10" t="s">
+      <c r="K4" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="L4" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="M4" s="10" t="s">
+      <c r="M4" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N4" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="N4" s="10" t="b">
+      <c r="O4" s="10" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
@@ -1181,40 +1245,43 @@
         <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>99</v>
-      </c>
-      <c r="E5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
         <v>11</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>12</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>27</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L5" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N5" s="4" t="b">
+      <c r="K5" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M5" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O5" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
@@ -1226,40 +1293,43 @@
         <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
         <v>11</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>12</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>30</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="J6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J6" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L6" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N6" s="4" t="b">
+      <c r="K6" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M6" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O6" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
@@ -1271,40 +1341,43 @@
         <v>32</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="E7" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="E7" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="G7" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="I7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="J7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="J7" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="K7" s="10" t="s">
+      <c r="K7" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="L7" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="M7" s="10" t="s">
+      <c r="M7" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="N7" s="10" t="b">
+      <c r="O7" s="10" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
@@ -1316,40 +1389,43 @@
         <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>102</v>
-      </c>
-      <c r="E8" t="s">
+        <v>101</v>
+      </c>
+      <c r="E8" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
         <v>11</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>12</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>36</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>14</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="J8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J8" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L8" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N8" s="4" t="b">
+      <c r="K8" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O8" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
@@ -1361,40 +1437,43 @@
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
-      </c>
-      <c r="E9" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
         <v>11</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>12</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>39</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="J9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L9" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N9" s="4" t="b">
+      <c r="K9" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O9" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
@@ -1402,813 +1481,865 @@
       <c r="B10" t="s">
         <v>40</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E10" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="G10" t="s">
         <v>42</v>
       </c>
-      <c r="F10" t="s">
+      <c r="H10" t="s">
         <v>43</v>
       </c>
-      <c r="G10" t="s">
-        <v>44</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>14</v>
       </c>
-      <c r="I10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J10" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L10" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N10" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="O10" s="4" t="s">
-        <v>108</v>
-      </c>
+      <c r="J10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K10" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" s="4"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
         <v>45</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E11" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E11" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" t="s">
-        <v>47</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>14</v>
       </c>
-      <c r="I11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J11" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L11" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N11" s="4" t="b">
+      <c r="J11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K11" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M11" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O11" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
         <v>48</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E12" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" t="s">
-        <v>50</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>14</v>
       </c>
-      <c r="I12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J12" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L12" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M12" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N12" s="4" t="b">
+      <c r="J12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K12" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M12" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O12" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" t="s">
         <v>51</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E13" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" t="s">
-        <v>53</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>14</v>
       </c>
-      <c r="I13" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J13" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L13" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M13" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N13" s="4" t="b">
+      <c r="J13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K13" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M13" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O13" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" t="s">
         <v>54</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E14" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" t="s">
+        <v>42</v>
+      </c>
+      <c r="H14" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E14" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" t="s">
-        <v>43</v>
-      </c>
-      <c r="G14" t="s">
-        <v>56</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>14</v>
       </c>
-      <c r="I14" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J14" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L14" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N14" s="4" t="b">
+      <c r="J14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K14" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M14" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O14" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B15" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="D15" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="E15" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="H15" s="8" t="s">
+      <c r="I15" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="I15" s="9" t="s">
+      <c r="J15" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="J15" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="K15" s="10" t="s">
+      <c r="K15" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="L15" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="M15" s="10" t="s">
+      <c r="M15" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="N15" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="N15" s="10" t="b">
+      <c r="O15" s="10" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" t="s">
         <v>60</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
+        <v>104</v>
+      </c>
+      <c r="E16" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" t="s">
         <v>61</v>
       </c>
-      <c r="D16" t="s">
-        <v>105</v>
-      </c>
-      <c r="E16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F16" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" t="s">
-        <v>62</v>
-      </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>14</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="J16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J16" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L16" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M16" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N16" s="4" t="b">
+      <c r="K16" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M16" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O16" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" t="s">
         <v>63</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E17" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" t="s">
+        <v>12</v>
+      </c>
+      <c r="H17" t="s">
         <v>64</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" t="s">
-        <v>12</v>
-      </c>
-      <c r="G17" t="s">
-        <v>65</v>
-      </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>14</v>
       </c>
-      <c r="I17" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J17" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K17" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L17" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M17" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N17" s="4" t="b">
+      <c r="J17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K17" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M17" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O17" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B18" t="s">
+        <v>65</v>
+      </c>
+      <c r="C18" t="s">
         <v>66</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E18" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" t="s">
+        <v>12</v>
+      </c>
+      <c r="H18" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E18" t="s">
-        <v>11</v>
-      </c>
-      <c r="F18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" t="s">
-        <v>68</v>
-      </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>14</v>
       </c>
-      <c r="I18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J18" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L18" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M18" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N18" s="4" t="b">
+      <c r="J18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K18" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M18" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O18" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B19" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" t="s">
         <v>69</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" t="s">
+        <v>12</v>
+      </c>
+      <c r="H19" t="s">
         <v>70</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E19" t="s">
-        <v>11</v>
-      </c>
-      <c r="F19" t="s">
-        <v>12</v>
-      </c>
-      <c r="G19" t="s">
-        <v>71</v>
-      </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>14</v>
       </c>
-      <c r="I19" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J19" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K19" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L19" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M19" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N19" s="4" t="b">
+      <c r="J19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K19" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M19" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N19" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O19" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B20" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" t="s">
         <v>72</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E20" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20" t="s">
+        <v>12</v>
+      </c>
+      <c r="H20" t="s">
         <v>73</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E20" t="s">
-        <v>11</v>
-      </c>
-      <c r="F20" t="s">
-        <v>12</v>
-      </c>
-      <c r="G20" t="s">
-        <v>74</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>14</v>
       </c>
-      <c r="I20" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J20" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K20" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L20" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M20" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N20" s="4" t="b">
+      <c r="J20" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K20" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M20" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N20" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O20" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B21" t="s">
+        <v>74</v>
+      </c>
+      <c r="C21" t="s">
         <v>75</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E21" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>11</v>
+      </c>
+      <c r="G21" t="s">
+        <v>12</v>
+      </c>
+      <c r="H21" t="s">
         <v>76</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E21" t="s">
-        <v>11</v>
-      </c>
-      <c r="F21" t="s">
-        <v>12</v>
-      </c>
-      <c r="G21" t="s">
-        <v>77</v>
-      </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>14</v>
       </c>
-      <c r="I21" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J21" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K21" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L21" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M21" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N21" s="4" t="b">
+      <c r="J21" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K21" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M21" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N21" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O21" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B22" t="s">
+        <v>77</v>
+      </c>
+      <c r="C22" t="s">
         <v>78</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E22" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F22" t="s">
+        <v>11</v>
+      </c>
+      <c r="G22" t="s">
+        <v>12</v>
+      </c>
+      <c r="H22" t="s">
         <v>79</v>
       </c>
-      <c r="D22" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E22" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" t="s">
-        <v>80</v>
-      </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>14</v>
       </c>
-      <c r="I22" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J22" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L22" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M22" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N22" s="4" t="b">
+      <c r="J22" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K22" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M22" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N22" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O22" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B23" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" t="s">
         <v>81</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E23" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" t="s">
+        <v>11</v>
+      </c>
+      <c r="G23" t="s">
+        <v>12</v>
+      </c>
+      <c r="H23" t="s">
         <v>82</v>
       </c>
-      <c r="D23" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E23" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" t="s">
-        <v>12</v>
-      </c>
-      <c r="G23" t="s">
-        <v>83</v>
-      </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>14</v>
       </c>
-      <c r="I23" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J23" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K23" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L23" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M23" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N23" s="4" t="b">
+      <c r="J23" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K23" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M23" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N23" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O23" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B24" t="s">
+        <v>83</v>
+      </c>
+      <c r="C24" t="s">
         <v>84</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E24" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" t="s">
+        <v>12</v>
+      </c>
+      <c r="H24" t="s">
         <v>85</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E24" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" t="s">
-        <v>86</v>
-      </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>14</v>
       </c>
-      <c r="I24" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J24" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K24" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L24" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M24" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N24" s="4" t="b">
+      <c r="J24" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K24" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M24" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N24" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O24" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B25" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C25" t="s">
         <v>87</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E25" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25" t="s">
+        <v>11</v>
+      </c>
+      <c r="G25" t="s">
+        <v>12</v>
+      </c>
+      <c r="H25" t="s">
         <v>88</v>
       </c>
-      <c r="D25" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E25" t="s">
-        <v>11</v>
-      </c>
-      <c r="F25" t="s">
-        <v>12</v>
-      </c>
-      <c r="G25" t="s">
-        <v>89</v>
-      </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>14</v>
       </c>
-      <c r="I25" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J25" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K25" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L25" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M25" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N25" s="4" t="b">
+      <c r="J25" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K25" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M25" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N25" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O25" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B26" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" t="s">
         <v>90</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E26" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>11</v>
+      </c>
+      <c r="G26" t="s">
+        <v>12</v>
+      </c>
+      <c r="H26" t="s">
         <v>91</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E26" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26" t="s">
-        <v>12</v>
-      </c>
-      <c r="G26" t="s">
-        <v>92</v>
-      </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>14</v>
       </c>
-      <c r="I26" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J26" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K26" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L26" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M26" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N26" s="4" t="b">
+      <c r="J26" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K26" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M26" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N26" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O26" s="4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="b">
         <f>IF(AND(Table1[[#This Row],[Groups Complete]],Table1[[#This Row],[License Complete]],Table1[[#This Row],[Device Complete]]),TRUE,FALSE)</f>
         <v>1</v>
       </c>
       <c r="B27" t="s">
+        <v>92</v>
+      </c>
+      <c r="C27" t="s">
         <v>93</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E27" s="13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F27" t="s">
+        <v>11</v>
+      </c>
+      <c r="G27" t="s">
+        <v>12</v>
+      </c>
+      <c r="H27" t="s">
         <v>94</v>
       </c>
-      <c r="D27" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E27" t="s">
-        <v>11</v>
-      </c>
-      <c r="F27" t="s">
-        <v>12</v>
-      </c>
-      <c r="G27" t="s">
-        <v>95</v>
-      </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>14</v>
       </c>
-      <c r="I27" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J27" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="K27" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="L27" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M27" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N27" s="4" t="b">
+      <c r="J27" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K27" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="M27" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N27" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O27" s="4" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:O27">
+  <conditionalFormatting sqref="A2:P27">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$A2</formula>
     </cfRule>

</xml_diff>